<commit_message>
Top 8: replace doctor-name string with best clinic string
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L2kGRjNiXDu5bVc35jPrtD
</commit_message>
<xml_diff>
--- a/Bloom_AI_Rank_Strings.xlsx
+++ b/Bloom_AI_Rank_Strings.xlsx
@@ -778,47 +778,47 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Dr Vinod Sonawane – beard / FUE hair transplant doctor in Mumbai</t>
+          <t>Best hair transplant clinic in Mumbai</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>hair transplant doctor mumbai / best hair transplant surgeon in mumbai / vin hair transplant (brand-adjacent)</t>
+          <t>best hair clinic mumbai (140, Pos 1) / best hair transplant clinic in mumbai / mumbai best hair transplant clinic (70)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Doctor entity (E-E-A-T)</t>
+          <t>Best-of (AI loves lists)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Dr Vinod Sonawane – Hair Transplant Surgeon, Mumbai (Physician schema)</t>
+          <t>Best Hair Transplant Clinic in Mumbai | Bloom (Andheri West &amp; Ghatkopar)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>70 + 20</t>
+          <t>140 + 70 + 10</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>AI engines recommend named doctors. Building a clear doctor entity (bio, credentials, sameAs links) is the quickest way to get named in answers.</t>
+          <t>Already Pos 1 for best hair clinic mumbai. AI engines answer best-clinic questions from reviews, lists and GBP, which we can build in 30 days.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Medium-Strong</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Very high</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Doctor page with Physician schema, qualifications, sameAs (Instagram, YouTube, GBP), media mentions, 3 expert Q&amp;As.</t>
+          <t>Clinic-focused page with 40-word answer box, comparison vs other options, 2 locations, review count, awards; get listed in top-10 articles; 15 new reviews; Quora + Reddit answers.</t>
         </is>
       </c>
     </row>
@@ -1094,17 +1094,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Best hair transplant clinic in Mumbai</t>
+          <t>Hair transplant clinic in Mumbai</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>hair transplant clinic mumbai / best hair clinic mumbai</t>
+          <t>hair transplant clinic mumbai (20) / hair transplant clinic in mumbai (10)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Best-of</t>
+          <t>Clinic</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -4176,27 +4176,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Dr Vinod Sonawane – beard / FUE hair transplant doctor in Mumbai</t>
+          <t>Best hair transplant clinic in Mumbai</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Which are the best clinics/doctors for: dr vinod sonawane – beard / fue hair transplant doctor in mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
+          <t>Which are the best clinics/doctors for: best hair transplant clinic in mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Using current web sources, list top recommendations for "dr vinod sonawane – beard / fue hair transplant doctor in mumbai" with citations.</t>
+          <t>Using current web sources, list top recommendations for "best hair transplant clinic in mumbai" with citations.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Honest experience with dr vinod sonawane – beard / fue hair transplant doctor in mumbai? Which clinic did you choose?</t>
+          <t>Honest experience with best hair transplant clinic in mumbai? Which clinic did you choose?</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>What is the best option for dr vinod sonawane – beard / fue hair transplant doctor in mumbai and why?</t>
+          <t>What is the best option for best hair transplant clinic in mumbai and why?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add search volume and est. time-to-rank (AI, SERP) columns
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L2kGRjNiXDu5bVc35jPrtD
</commit_message>
<xml_diff>
--- a/Bloom_AI_Rank_Strings.xlsx
+++ b/Bloom_AI_Rank_Strings.xlsx
@@ -555,19 +555,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -583,40 +586,55 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Keyword search volume (monthly)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Estimated time to rank on AI</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Estimated time to rank on SERP (Google)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Keyword-data source</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Page / content to build</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Monthly volume (tool)</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Volume detail (tool)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Why this one</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Chance of AI visibility in 30 days*</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Lead value</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>What we will do (actions)</t>
         </is>
@@ -631,42 +649,55 @@
           <t>Hair transplant in Andheri West</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Already #1 - maintain</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>hair transplant in andheri west / hair transplant andheri west</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Local + clinic (main)</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Hair Transplant in Andheri West, Mumbai | Bloom Hair Transplant</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>50 (Pos 1 already)</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Already ranks #1 in Google. Clinic is physically there, so Google Business Profile + reviews make AI engines name Bloom for this location.</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>High (ready-to-book)</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Add 'Hair transplant in Andheri West' H1 + 40-word answer box + FAQPage + MedicalClinic schema; 10 reviews mentioning Andheri West; GBP posts; Quora + Reddit answers.</t>
         </is>
@@ -681,42 +712,55 @@
           <t>Hair transplant doctor in Ghatkopar / hair specialist in Ghatkopar</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>3-6 weeks</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>hair specialist in ghatkopar</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Local + clinic (2nd)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>NEW PAGE: Hair Transplant Clinic in Ghatkopar East</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Very low competition, Bloom has 2nd clinic there, almost no one else answers this. Fastest realistic AI win.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Very strong</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Create Ghatkopar page with address, map, doctor, timings, FAQ; GBP for Ghatkopar; NAP citations; 5 reviews naming Ghatkopar.</t>
         </is>
@@ -731,42 +775,55 @@
           <t>Female hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>female hair transplant in mumbai / female hair trasnplant mumbai</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Niche (low competition)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Female Hair Transplant in Mumbai | Bloom</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Difficulty only 14, competition 0.08. Service exists on site. AI answers for female hair loss have few good sources.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Very strong</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>High (high-value patients)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Dedicated page + PCOS / postpartum / thinning FAQs; doctor-authored article; Quora answers; female patient story (with consent).</t>
         </is>
@@ -781,42 +838,55 @@
           <t>Best hair transplant clinic in Mumbai</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Already #1 - maintain; variants 2-3 months</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>best hair clinic mumbai (140, Pos 1) / best hair transplant clinic in mumbai / mumbai best hair transplant clinic (70)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Best-of (AI loves lists)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Best Hair Transplant Clinic in Mumbai | Bloom (Andheri West &amp; Ghatkopar)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>140 + 70 + 10</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Already Pos 1 for best hair clinic mumbai. AI engines answer best-clinic questions from reviews, lists and GBP, which we can build in 30 days.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Medium-Strong</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Very high</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Clinic-focused page with 40-word answer box, comparison vs other options, 2 locations, review count, awards; get listed in top-10 articles; 15 new reviews; Quora + Reddit answers.</t>
         </is>
@@ -831,42 +901,55 @@
           <t>Failed / repair hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>not in tool – supporting: hair restoration mumbai (20) + repair intent</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Niche (low competition)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Hair Transplant Repair &amp; Revision in Mumbai</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>~20 (est.)</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Few clinics answer 'my transplant failed' properly; patients ask AI this and are high-intent. Easy to be the cited source.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Strong</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Very high</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Repair page, before/after cases (with consent), 'why transplants fail' guide, FAQ schema.</t>
         </is>
@@ -881,42 +964,55 @@
           <t>Hair transplant cost in Mumbai</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>4-6 weeks</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks (already Pos 4 for low cost)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>cheap hair transplant in mumbai (20) / hair transplant in mumbai low cost (10, Pos 4)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Money / lead intent</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Hair Transplant Cost in Mumbai – Price per Graft (2026)</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>30 + 10 (AI asks far more)</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Already Pos 4 for low cost. Cost questions are asked in ChatGPT constantly; answer with real ranges + factors to get cited.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Strong (needs client price range)</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Very high</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Cost page with price/graft range, factors table, EMI, FAQ; client must confirm numbers.</t>
         </is>
@@ -931,42 +1027,55 @@
           <t>FUE vs FUT vs DHI – which hair transplant is best in Mumbai</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="4" t="n">
+        <v>260</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>3-6 weeks</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>fue hair transplant in mumbai (260) / dhi hair transplant in mumbai (10) / fut hair transplant in mumbai (Pos 1)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Comparison (AI loves)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>FUE vs DHI vs FUT: Which Is Right for You?</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>260 + 10 + 10</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Comparison tables are the most-cited format in AI answers. FUE vol 260; FUT already Pos 1.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Very strong</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Medium-High</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Comparison table, 40-word verdict, FAQ, video embed; internal link to each type page.</t>
         </is>
@@ -981,54 +1090,75 @@
           <t>Celebrity hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>celebrity hair transplant in mumbai</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Authority / trust</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Celebrity Hair Transplant in Mumbai – Bloom</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>90 (Pos 12)</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>Site already shows celebrity photos; 'celebrity' + Mumbai has only 0.49 competition. Boosts brand mentions in AI.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Medium-Strong</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Medium (trust builder)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Media/celebrity page with consent-verified claims, Mid-Day/press links, schema; PR mentions.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Time estimates are planning guidelines (assuming pages are published in week 1-2), not guarantees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Assessment, not a guarantee. AI engines change answers daily. See Client Wording sheet.</t>
         </is>
@@ -1045,15 +1175,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1069,20 +1202,35 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Keyword-data reference (volume)</t>
+          <t>Keyword search volume (monthly)</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>Estimated time to rank on AI</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Estimated time to rank on SERP (Google)</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Keyword-data reference</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Goal</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
@@ -1097,22 +1245,35 @@
           <t>Hair transplant clinic in Mumbai</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>hair transplant clinic mumbai (20) / hair transplant clinic in mumbai (10)</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Clinic</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Ranking, trust</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1127,22 +1288,35 @@
           <t>Best hair transplant doctor in Mumbai</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>best hair transplant doctor in mumbai</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Best-of</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Ranking, trust</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1157,22 +1331,35 @@
           <t>Best hair transplant surgeon in Mumbai</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>10-14 weeks</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>best hair transplant surgeon in mumbai (70)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Best-of</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1187,22 +1374,35 @@
           <t>Top 10 hair transplant clinics in Mumbai</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>10-16 weeks</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>top 10 hair transplant clinic in mumbai (110)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>List</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Ranking (AI cites lists)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1217,22 +1417,35 @@
           <t>Hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="n">
+        <v>1900</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>12-24 weeks</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>16-24 weeks</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>hair transplantation mumbai (1900)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Head term</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Ranking (long term)</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1247,22 +1460,35 @@
           <t>Hair transplant cost in Mumbai per graft</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>4-6 weeks</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>hair transplant cost mumbai</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1277,22 +1503,35 @@
           <t>Is hair transplant painful? Recovery time</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>does hair transplant has any side effects (20)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Leads, AI answers</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1307,22 +1546,35 @@
           <t>Hair transplant side effects</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>hair transplant surgery side effects (10, Pos 1)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>AI answers</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1339,20 +1591,35 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>AI answers</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1367,22 +1634,35 @@
           <t>FUE hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="4" t="n">
+        <v>260</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>fue hair transplant in mumbai (260)</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Technique</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Ranking + leads</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1397,22 +1677,35 @@
           <t>Best FUE hair transplant clinic in Mumbai</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>3-6 weeks</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>fue hair transplant clinic in mumbai (Pos 1)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Technique</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1427,22 +1720,35 @@
           <t>DHI hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>3-6 weeks</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>dhi hair transplant in mumbai (10)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Technique</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1457,22 +1763,35 @@
           <t>Robotic hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>robotic hair transplant in mumbai (10, Pos 1)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Technique</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Ranking (already Pos 1)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1489,20 +1808,35 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1519,20 +1853,35 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1547,22 +1896,35 @@
           <t>Hair transplant for PCOS</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>hair transplant for pcos (10, Pos 1)</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Leads (already Pos 1)</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1577,22 +1939,35 @@
           <t>Hair loss in women: causes and treatment</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>hair loss due to hormones (50, Pos 1)</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>AI answers, leads</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1607,22 +1982,35 @@
           <t>Hair transplant in Bandra</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>hair transplant bandra (90)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1637,22 +2025,35 @@
           <t>Hair transplant in South Mumbai</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>hair transplant in south mumbai (Pos 1)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1667,22 +2068,35 @@
           <t>Hair transplant in Mulund / Thane / Navi Mumbai</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>hair transplant in mulund (10)</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1699,20 +2113,35 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>3-6 weeks</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Leads (GBP)</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1727,22 +2156,35 @@
           <t>Hair specialist in Mumbai</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>10-16 weeks</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>12-20 weeks</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>hair specialist in mumbai (590)</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Doctor</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1757,22 +2199,35 @@
           <t>Best hair doctor in Mumbai</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="4" t="n">
+        <v>590</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>best hair doctor in mumbai (590, Pos 1)</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Doctor</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Ranking (Pos 1 already)</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1787,22 +2242,35 @@
           <t>Hair treatment in Mumbai (PRP, mesotherapy)</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="4" t="n">
+        <v>480</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>10-16 weeks</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>hair treatment in mumbai (480)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Treatment</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1817,22 +2285,35 @@
           <t>Scalp micropigmentation in Mumbai</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>scalp micropigmentation mumbai (70)</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Leads (only if offered)</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1847,22 +2328,35 @@
           <t>Hair restoration in Mumbai</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>8-12 weeks</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>hair restoration mumbai (20)</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Head term</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1877,22 +2371,35 @@
           <t>Cheap / affordable hair transplant in Mumbai</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>cheap hair transplant in mumbai (20)</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1909,20 +2416,35 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>4-6 weeks</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>6-10 weeks</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Proof</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>Trust, leads</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1939,20 +2461,35 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
+          <t>Not in tool</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>3-5 weeks</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>4-8 weeks</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>AI answers</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
         </is>
@@ -1967,24 +2504,45 @@
           <t>What causes hair loss in early 20s</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Already Pos 1 - maintain</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>what causes hair loss in early 20s (10, Pos 1)</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>AI answers, top-funnel</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Create/optimise a section or blog + FAQ schema; link to Top-8 page; answer on Quora/Reddit</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Time estimates are planning guidelines (assuming pages are published in week 1-2), not guarantees. Volume = monthly searches from the Semrush-style table; 'Not in tool' = no data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use clean Title Case keyword strings like the first research sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L2kGRjNiXDu5bVc35jPrtD
</commit_message>
<xml_diff>
--- a/Bloom_AI_Rank_Strings.xlsx
+++ b/Bloom_AI_Rank_Strings.xlsx
@@ -646,7 +646,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in Andheri West</t>
+          <t>Hair Transplant In Andheri West</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
@@ -709,7 +709,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant doctor in Ghatkopar / hair specialist in Ghatkopar</t>
+          <t>Hair Specialist In Ghatkopar</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Female hair transplant in Mumbai</t>
+          <t>Female Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
@@ -835,7 +835,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Best hair transplant clinic in Mumbai</t>
+          <t>Best Hair Transplant Clinic In Mumbai</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -898,7 +898,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Failed / repair hair transplant in Mumbai</t>
+          <t>Failed Hair Transplant Repair In Mumbai</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -961,7 +961,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant cost in Mumbai</t>
+          <t>Hair Transplant Cost In Mumbai</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>FUE vs FUT vs DHI – which hair transplant is best in Mumbai</t>
+          <t>FUE Vs FUT Vs DHI Hair Transplant Mumbai</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Celebrity hair transplant in Mumbai</t>
+          <t>Celebrity Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant clinic in Mumbai</t>
+          <t>Hair Transplant Clinic In Mumbai</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Best hair transplant doctor in Mumbai</t>
+          <t>Best Hair Transplant Doctor In Mumbai</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Best hair transplant surgeon in Mumbai</t>
+          <t>Best Hair Transplant Surgeon In Mumbai</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Top 10 hair transplant clinics in Mumbai</t>
+          <t>Top 10 Hair Transplant Clinics In Mumbai</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in Mumbai</t>
+          <t>Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant cost in Mumbai per graft</t>
+          <t>Hair Transplant Cost Per Graft In Mumbai</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Is hair transplant painful? Recovery time</t>
+          <t>Hair Transplant Recovery Time</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant side effects</t>
+          <t>Hair Transplant Side Effects</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant results timeline month by month</t>
+          <t>Hair Transplant Results Timeline</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>FUE hair transplant in Mumbai</t>
+          <t>FUE Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Best FUE hair transplant clinic in Mumbai</t>
+          <t>Best FUE Hair Transplant Clinic In Mumbai</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>DHI hair transplant in Mumbai</t>
+          <t>DHI Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Robotic hair transplant in Mumbai</t>
+          <t>Robotic Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Beard transplant in Mumbai</t>
+          <t>Beard Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Eyebrow transplant in Mumbai</t>
+          <t>Eyebrow Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant for PCOS</t>
+          <t>Hair Transplant For PCOS</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Hair loss in women: causes and treatment</t>
+          <t>Hair Loss In Women Treatment</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in Bandra</t>
+          <t>Hair Transplant In Bandra</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in South Mumbai</t>
+          <t>Hair Transplant In South Mumbai</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in Mulund / Thane / Navi Mumbai</t>
+          <t>Hair Transplant In Mulund</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant clinic near me (Andheri / Ghatkopar)</t>
+          <t>Hair Transplant Clinic Near Me</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Hair specialist in Mumbai</t>
+          <t>Hair Specialist In Mumbai</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Best hair doctor in Mumbai</t>
+          <t>Best Hair Doctor In Mumbai</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Hair treatment in Mumbai (PRP, mesotherapy)</t>
+          <t>Hair Treatment In Mumbai</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Scalp micropigmentation in Mumbai</t>
+          <t>Scalp Micropigmentation In Mumbai</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Hair restoration in Mumbai</t>
+          <t>Hair Restoration In Mumbai</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Cheap / affordable hair transplant in Mumbai</t>
+          <t>Cheap Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant before and after (Mumbai results)</t>
+          <t>Hair Transplant Before And After Mumbai</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Best age for hair transplant / who is a good candidate</t>
+          <t>Best Age For Hair Transplant</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>What causes hair loss in early 20s</t>
+          <t>Hair Loss In Early 20s Causes</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -4653,7 +4653,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant in Andheri West</t>
+          <t>Hair Transplant In Andheri West</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -4680,34 +4680,34 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant doctor in Ghatkopar / hair specialist in Ghatkopar</t>
+          <t>Hair Specialist In Ghatkopar</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Which are the best clinics/doctors for: hair transplant doctor in ghatkopar / hair specialist in ghatkopar? Include clinic name, doctor, location, cost range and reviews.</t>
+          <t>Which are the best clinics/doctors for: hair specialist in ghatkopar? Include clinic name, doctor, location, cost range and reviews.</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Using current web sources, list top recommendations for "hair transplant doctor in ghatkopar / hair specialist in ghatkopar" with citations.</t>
+          <t>Using current web sources, list top recommendations for "hair specialist in ghatkopar" with citations.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Honest experience with hair transplant doctor in ghatkopar / hair specialist in ghatkopar? Which clinic did you choose?</t>
+          <t>Honest experience with hair specialist in ghatkopar? Which clinic did you choose?</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>What is the best option for hair transplant doctor in ghatkopar / hair specialist in ghatkopar and why?</t>
+          <t>What is the best option for hair specialist in ghatkopar and why?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Female hair transplant in Mumbai</t>
+          <t>Female Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -4734,7 +4734,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Best hair transplant clinic in Mumbai</t>
+          <t>Best Hair Transplant Clinic In Mumbai</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -4761,34 +4761,34 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Failed / repair hair transplant in Mumbai</t>
+          <t>Failed Hair Transplant Repair In Mumbai</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Which are the best clinics/doctors for: failed / repair hair transplant in mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
+          <t>Which are the best clinics/doctors for: failed hair transplant repair in mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Using current web sources, list top recommendations for "failed / repair hair transplant in mumbai" with citations.</t>
+          <t>Using current web sources, list top recommendations for "failed hair transplant repair in mumbai" with citations.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Honest experience with failed / repair hair transplant in mumbai? Which clinic did you choose?</t>
+          <t>Honest experience with failed hair transplant repair in mumbai? Which clinic did you choose?</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>What is the best option for failed / repair hair transplant in mumbai and why?</t>
+          <t>What is the best option for failed hair transplant repair in mumbai and why?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Hair transplant cost in Mumbai</t>
+          <t>Hair Transplant Cost In Mumbai</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -4815,34 +4815,34 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>FUE vs FUT vs DHI – which hair transplant is best in Mumbai</t>
+          <t>FUE Vs FUT Vs DHI Hair Transplant Mumbai</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Which are the best clinics/doctors for: fue vs fut vs dhi – which hair transplant is best in mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
+          <t>Which are the best clinics/doctors for: fue vs fut vs dhi hair transplant mumbai? Include clinic name, doctor, location, cost range and reviews.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Using current web sources, list top recommendations for "fue vs fut vs dhi – which hair transplant is best in mumbai" with citations.</t>
+          <t>Using current web sources, list top recommendations for "fue vs fut vs dhi hair transplant mumbai" with citations.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Honest experience with fue vs fut vs dhi – which hair transplant is best in mumbai? Which clinic did you choose?</t>
+          <t>Honest experience with fue vs fut vs dhi hair transplant mumbai? Which clinic did you choose?</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>What is the best option for fue vs fut vs dhi – which hair transplant is best in mumbai and why?</t>
+          <t>What is the best option for fue vs fut vs dhi hair transplant mumbai and why?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Celebrity hair transplant in Mumbai</t>
+          <t>Celebrity Hair Transplant In Mumbai</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">

</xml_diff>